<commit_message>
new ordering for automation
</commit_message>
<xml_diff>
--- a/sim_output.xlsx
+++ b/sim_output.xlsx
@@ -1125,13 +1125,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4015E8FE-8E7F-427D-8B12-B707FCD4DE83}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AB58F530-E1E8-4FC7-B276-828D5709F7E8}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F115D9B2-40BD-43BD-9ECD-9B48C69431D0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{823E1D5D-A5B7-4D0C-B39A-D39844A8E9A2}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB8C82F1-1839-4A92-9955-C837ABF00F64}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{84A76BE7-49D0-4645-A396-4BA1D305ACB8}"/>
 </file>
</xml_diff>